<commit_message>
refactor: resolve eslint errors and deduplicate todo list logic
</commit_message>
<xml_diff>
--- a/연차정정_및_소급대상자_명단.xlsx
+++ b/연차정정_및_소급대상자_명단.xlsx
@@ -397,22 +397,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData/>
+  <dimension ref="A1:H7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>직원명</v>
+      </c>
+      <c r="B1" t="str">
+        <v>입사일</v>
+      </c>
+      <c r="C1" t="str">
+        <v>근속 기간</v>
+      </c>
+      <c r="D1" t="str">
+        <v>소급 월차(개)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>총 발생 연차</v>
+      </c>
+      <c r="F1" t="str">
+        <v>누적 사용</v>
+      </c>
+      <c r="G1" t="str">
+        <v>누적 소멸</v>
+      </c>
+      <c r="H1" t="str">
+        <v>최종 잔여 연차</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>이가연</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2023-09-08</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2년 9개월</v>
+      </c>
+      <c r="D2" t="str">
+        <v>11 개</v>
+      </c>
+      <c r="E2" t="str">
+        <v>41.0 일</v>
+      </c>
+      <c r="F2" t="str">
+        <v>22.0 일</v>
+      </c>
+      <c r="G2" t="str">
+        <v>11.0 일</v>
+      </c>
+      <c r="H2" t="str">
+        <v>8.0 일</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>김수지</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2023-09-20</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2년 9개월</v>
+      </c>
+      <c r="D3" t="str">
+        <v>11 개</v>
+      </c>
+      <c r="E3" t="str">
+        <v>41.0 일</v>
+      </c>
+      <c r="F3" t="str">
+        <v>15.0 일</v>
+      </c>
+      <c r="G3" t="str">
+        <v>11.0 일</v>
+      </c>
+      <c r="H3" t="str">
+        <v>15.0 일</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>홍자비</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2023-10-24</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2년 8개월</v>
+      </c>
+      <c r="D4" t="str">
+        <v>11 개</v>
+      </c>
+      <c r="E4" t="str">
+        <v>41.0 일</v>
+      </c>
+      <c r="F4" t="str">
+        <v>13.0 일</v>
+      </c>
+      <c r="G4" t="str">
+        <v>11.0 일</v>
+      </c>
+      <c r="H4" t="str">
+        <v>17.0 일</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>조현준</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2024-06-03</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2년 0개월</v>
+      </c>
+      <c r="D5" t="str">
+        <v>11 개</v>
+      </c>
+      <c r="E5" t="str">
+        <v>26.0 일</v>
+      </c>
+      <c r="F5" t="str">
+        <v>12.0 일</v>
+      </c>
+      <c r="G5" t="str">
+        <v>11.0 일</v>
+      </c>
+      <c r="H5" t="str">
+        <v>3.0 일</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>송소현</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2025-01-03</v>
+      </c>
+      <c r="C6" t="str">
+        <v>1년 5개월</v>
+      </c>
+      <c r="D6" t="str">
+        <v>11 개</v>
+      </c>
+      <c r="E6" t="str">
+        <v>26.0 일</v>
+      </c>
+      <c r="F6" t="str">
+        <v>8.5 일</v>
+      </c>
+      <c r="G6" t="str">
+        <v>11.0 일</v>
+      </c>
+      <c r="H6" t="str">
+        <v>6.5 일</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>박지연</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2025-10-30</v>
+      </c>
+      <c r="C7" t="str">
+        <v>0년 8개월</v>
+      </c>
+      <c r="D7" t="str">
+        <v>1 개</v>
+      </c>
+      <c r="E7" t="str">
+        <v>8.0 일</v>
+      </c>
+      <c r="F7" t="str">
+        <v>0.0 일</v>
+      </c>
+      <c r="G7" t="str">
+        <v>0.0 일</v>
+      </c>
+      <c r="H7" t="str">
+        <v>8.0 일</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>